<commit_message>
Add DB3 pipeline outputs for 2013–2016
Each year's Output/<year>/ folder contains the full chain of intermediate
files (extracted, with_ids, geo_validated, …) plus the final deliverable:

  db3_<year>_FINAL.xlsx  →  Clean_Data | Removed_Rows | Summary_Report

2016 summary (first completed run with DS2 audit verification):
  - 84 clean rows, 4 removed rows, 251 PIPL total
  - All route totals reconcile with DS2 observer summaries where DS2 data exists
  - Removed: 2 Outback Key DS3 rows (unresolvable GPS) +
             2 Three Rooker Bar north island DS3 rows (group # recording error)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3/Output/2013/db3_2013_FINAL.xlsx
+++ b/Databases/Database3/Output/2013/db3_2013_FINAL.xlsx
@@ -1425,7 +1425,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-31 11:38</t>
+          <t>2026-04-18 12:14</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Route, Latitude, Longitude, SurveyDate, TotalObserved, FlagCode</t>
+          <t>Route, Latitude, Longitude, SurveyDate, TotalObserved, FlagCode, FlagColor, BandCombo</t>
         </is>
       </c>
     </row>

</xml_diff>